<commit_message>
feat: agregar hoja REL_REPORTES al template de layouts
</commit_message>
<xml_diff>
--- a/public/template_layouts_bajaware.xlsx
+++ b/public/template_layouts_bajaware.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LAYOUT" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CATALOGOS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REL_REPORTES" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +54,24 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +98,23 @@
         <fgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -106,11 +138,25 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -129,6 +175,18 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -776,4 +834,73 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>RELACIÓN LAYOUT → REPORTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>NOMBRE_CAMPO = campo del layout  |  USO = CLAVE_REP_GENERAL del reporte que lo usa  |  COLUMNA = posición en el reporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>NOMBRE_CAMPO</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>COLUMNA_REPORTE_APLICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>NOMBRE_CAMPO_EJEMPLO</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>CLAVE_REP_GENERAL_REPORTE</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>